<commit_message>
refactor(parser): replace recursive descent with LL(1) table driver
</commit_message>
<xml_diff>
--- a/实验设计/语法分析/语法表格/FIRST与FOLLOW表.xlsx
+++ b/实验设计/语法分析/语法表格/FIRST与FOLLOW表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIRST与FOLLOW" sheetId="1" r:id="R45a803247b0c40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIRST与FOLLOW" sheetId="1" r:id="Rc0923a929c794de3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1124,7 +1124,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28854f8303b547b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb7a0447db2a422a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>